<commit_message>
Datos al 16-10-2026, regiones de Base Instalada desde Cartera ST, mapas fijos y ajustes de visitas
- Base Instalada: los clientes que la hoja trae sin región toman la que dedujo la Cartera ST
  (CESFAM Constitución, Hospital del Salvador, Hospital Regional de Arica) y se mueven en los
  resúmenes por región; regiones completadas a mano en BI_clientes_sin_region.xlsx (14-10).
- Visitas: el extractor reconoce a Cristián Pérez aunque la hoja lo escriba «Cristian Perez Farias»;
  alias y región para 4 clientes de las visitas programadas que quedaban sin región.
- Mapas de Cartera de Clientes y de Visitas Ejecutivos quedan fijos bajo la barra al hacer scroll.
- EERR: vista «EERR limpio» y exportable (cambios de hoja_eerr.js).
- Datos actualizados al 16-10-2026 y presentación 19-10-2026.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BI_clientes_sin_region.xlsx
+++ b/BI_clientes_sin_region.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Cristian.Vera\Downloads\Panel-TECSERVICE\Panel-TECSERVICE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{363DCA76-B04C-4AB5-B6F1-91342ABE9A9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17941763-72DB-40D5-8F18-C2FCC81C4281}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20610" yWindow="-3045" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Clientes sin región" sheetId="1" r:id="rId1"/>
     <sheet name="Regiones" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029" iterate="1" calcOnSave="0"/>
+  <calcPr calcId="191029" calcCompleted="0" calcOnSave="0"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="799" uniqueCount="380">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="813" uniqueCount="380">
   <si>
     <t>Cliente</t>
   </si>
@@ -1183,7 +1183,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1201,6 +1201,14 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1235,7 +1243,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1246,6 +1254,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1267,11 +1276,8 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="BISinRegion" displayName="BISinRegion" ref="A1:H199">
   <autoFilter ref="A1:H199" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="ALEJANDRA SEPULVEDA"/>
-        <filter val="JOSE ALEJANDRO GONZALEZ"/>
-      </filters>
+    <filterColumn colId="7">
+      <filters blank="1"/>
     </filterColumn>
   </autoFilter>
   <tableColumns count="8">
@@ -1595,7 +1601,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H199"/>
+  <dimension ref="A1:L199"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="58" customWidth="1"/>
@@ -1632,7 +1638,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -1648,7 +1654,9 @@
       <c r="F2" t="s">
         <v>9</v>
       </c>
-      <c r="H2" s="4"/>
+      <c r="H2" s="4" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -2047,7 +2055,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="20" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>45</v>
       </c>
@@ -2066,7 +2074,9 @@
       <c r="F20" t="s">
         <v>9</v>
       </c>
-      <c r="H20" s="4"/>
+      <c r="H20" s="4" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="21" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
@@ -3214,7 +3224,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>144</v>
       </c>
@@ -3502,7 +3512,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="81" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>164</v>
       </c>
@@ -3525,7 +3535,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="82" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>166</v>
       </c>
@@ -3548,7 +3558,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="83" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>168</v>
       </c>
@@ -3571,7 +3581,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="84" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>170</v>
       </c>
@@ -3594,7 +3604,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="85" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>172</v>
       </c>
@@ -3617,7 +3627,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="86" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>174</v>
       </c>
@@ -3640,7 +3650,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="87" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>176</v>
       </c>
@@ -3656,9 +3666,12 @@
       <c r="F87" t="s">
         <v>9</v>
       </c>
-      <c r="H87" s="4"/>
-    </row>
-    <row r="88" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H87" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="L87" s="8"/>
+    </row>
+    <row r="88" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>177</v>
       </c>
@@ -3681,7 +3694,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="89" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>179</v>
       </c>
@@ -3701,7 +3714,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="90" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="6" t="s">
         <v>180</v>
       </c>
@@ -3724,7 +3737,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="91" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>182</v>
       </c>
@@ -3747,7 +3760,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="92" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>184</v>
       </c>
@@ -3770,7 +3783,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="93" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>186</v>
       </c>
@@ -3786,9 +3799,11 @@
       <c r="F93" t="s">
         <v>9</v>
       </c>
-      <c r="H93" s="4"/>
-    </row>
-    <row r="94" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H93" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="94" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>187</v>
       </c>
@@ -3811,7 +3826,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="95" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>189</v>
       </c>
@@ -3834,7 +3849,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="96" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>191</v>
       </c>
@@ -4133,7 +4148,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="109" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>216</v>
       </c>
@@ -4149,7 +4164,9 @@
       <c r="F109" t="s">
         <v>9</v>
       </c>
-      <c r="H109" s="4"/>
+      <c r="H109" s="4" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="110" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
@@ -4494,7 +4511,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="125" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>245</v>
       </c>
@@ -4510,9 +4527,11 @@
       <c r="F125" t="s">
         <v>9</v>
       </c>
-      <c r="H125" s="4"/>
-    </row>
-    <row r="126" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H125" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="126" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>246</v>
       </c>
@@ -4531,9 +4550,11 @@
       <c r="F126" t="s">
         <v>9</v>
       </c>
-      <c r="H126" s="5"/>
-    </row>
-    <row r="127" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H126" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="127" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>248</v>
       </c>
@@ -4549,7 +4570,9 @@
       <c r="F127" t="s">
         <v>9</v>
       </c>
-      <c r="H127" s="4"/>
+      <c r="H127" s="4" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="128" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
@@ -4597,7 +4620,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="130" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>253</v>
       </c>
@@ -4613,7 +4636,9 @@
       <c r="F130" t="s">
         <v>9</v>
       </c>
-      <c r="H130" s="4"/>
+      <c r="H130" s="4" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="131" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
@@ -4701,7 +4726,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="135" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>260</v>
       </c>
@@ -4720,9 +4745,11 @@
       <c r="F135" t="s">
         <v>9</v>
       </c>
-      <c r="H135" s="4"/>
-    </row>
-    <row r="136" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H135" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="136" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>262</v>
       </c>
@@ -4738,7 +4765,9 @@
       <c r="F136" t="s">
         <v>9</v>
       </c>
-      <c r="H136" s="4"/>
+      <c r="H136" s="4" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="137" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
@@ -5257,7 +5286,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="160" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>304</v>
       </c>
@@ -5707,7 +5736,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="180" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>338</v>
       </c>
@@ -5723,7 +5752,9 @@
       <c r="F180" t="s">
         <v>9</v>
       </c>
-      <c r="H180" s="4"/>
+      <c r="H180" s="4" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="181" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
@@ -5797,7 +5828,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="184" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>345</v>
       </c>
@@ -5813,7 +5844,9 @@
       <c r="F184" t="s">
         <v>9</v>
       </c>
-      <c r="H184" s="4"/>
+      <c r="H184" s="4" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="185" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
@@ -6135,7 +6168,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="199" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>371</v>
       </c>
@@ -6151,12 +6184,15 @@
       <c r="F199" t="s">
         <v>9</v>
       </c>
-      <c r="H199" s="4"/>
+      <c r="H199" s="4" t="s">
+        <v>12</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">

</xml_diff>